<commit_message>
Cranes and new 32xmap
</commit_message>
<xml_diff>
--- a/server/col-bit-masks.xlsx
+++ b/server/col-bit-masks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\IslesAssault\server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE5FAA98-3B2A-4622-B59F-98B37AB260A0}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F10515F-4941-466D-91B1-1F6EEDEB7D72}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{2BCF002E-063A-4B93-AEF0-3852F43F3447}"/>
   </bookViews>
@@ -51,9 +51,6 @@
     <t>OnGround(tanks, cars)</t>
   </si>
   <si>
-    <t>S, B, C, ground/water veh</t>
-  </si>
-  <si>
     <t>Air</t>
   </si>
   <si>
@@ -93,13 +90,16 @@
     <t>111011</t>
   </si>
   <si>
-    <t>S, ground/water veh</t>
-  </si>
-  <si>
     <t>001011</t>
   </si>
   <si>
     <t>000000</t>
+  </si>
+  <si>
+    <t>S, ground</t>
+  </si>
+  <si>
+    <t>S, B, C, ground</t>
   </si>
 </sst>
 </file>
@@ -506,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B925E8F-2FC1-4554-A761-C51717D7748F}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.28515625" style="1" customWidth="1"/>
@@ -542,17 +542,17 @@
         <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" s="3">
         <f>_xlfn.DECIMAL(B2,2)</f>
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F2" s="3">
         <f>_xlfn.DECIMAL(E2,2)</f>
@@ -564,88 +564,88 @@
         <v>7</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" s="3">
         <f>_xlfn.DECIMAL(B3,2)</f>
         <v>2</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F3" s="3">
-        <f t="shared" ref="F3:F7" si="0">_xlfn.DECIMAL(E3,2)</f>
+        <f t="shared" ref="F3:F4" si="0">_xlfn.DECIMAL(E3,2)</f>
         <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" s="3">
         <f>_xlfn.DECIMAL(B4,2)</f>
         <v>4</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F4" s="3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="3">
-        <f t="shared" ref="C5:C7" si="1">_xlfn.DECIMAL(B5,2)</f>
-        <v>8</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C6" s="3">
-        <f t="shared" si="1"/>
-        <v>16</v>
+        <f t="shared" ref="C6:C8" si="1">_xlfn.DECIMAL(B6,2)</f>
+        <v>8</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C7" s="3">
         <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="3">
+        <f t="shared" si="1"/>
         <v>32</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>20</v>
+      <c r="D8" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>